<commit_message>
Product #10 video V1.1: framing/readability corrections only
- Capture copies widen only the columns whose header text is clipped at the
  shipped width (view-only; 0 differing values vs the packaged workbook),
  captured at 960 dpi; all Rent Tracker headers in view now read in full.
- Header row never clipped at the card top; white margin past the table's
  right edge; Total Paid column dropped from balance scenes to keep phone
  text size. Story, timing, captions, values, rings, chips, end card kept.
- Engine: 4-sided canvas_pad; must_show validation (region stays in frame
  for the whole camera move) surfaced in QA.
- QA PASS 108/0/0: no white flash, no ghosting, no internal labels.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Je8YSkF1eYHDKU2du3MKbu
</commit_message>
<xml_diff>
--- a/video-engine/sources/p10-rental-property/capture/states/p10_after.xlsx
+++ b/video-engine/sources/p10-rental-property/capture/states/p10_after.xlsx
@@ -3275,21 +3275,21 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="22" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>

</xml_diff>